<commit_message>
Add correcao-de-cargas to Ferramentas Gerais
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -617,6 +617,28 @@
       <c r="D7" s="3" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/aquickreportofseismographicdata/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>correcao-de-cargas</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Correção de Cargas</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/correcao-de-cargas</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/correcao-de-cargas/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add analisador-de-sismograma to general tools
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -623,20 +623,42 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>analisador-de-sismograma</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Analisador de Sismograma - Waveform</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/analisador-de-sismograma</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/analisador-de-sismograma/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>correcao-de-cargas</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Correção de Cargas</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>https://github.com/SILVAThiagoFerreira/correcao-de-cargas</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/correcao-de-cargas/</t>
         </is>

</xml_diff>